<commit_message>
fix(seguridad): sanitizar rutas absolutas en artefactos
</commit_message>
<xml_diff>
--- a/08-qa-uat/matriz-ejecucion.xlsx
+++ b/08-qa-uat/matriz-ejecucion.xlsx
@@ -567,7 +567,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29T01:51:55-03:00</t>
+          <t>2026-10-29T02:16:36-03:00</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Windows 11; Python 3.15.0; base C:/Users/User/Documents/nova-payments-aml/05-core-middleware/db/novabank.db; pytest 204 pruebas</t>
+          <t>Windows 11; Python 3.15.0; base 05-core-middleware/db/novabank.db; pytest 204 pruebas</t>
         </is>
       </c>
     </row>
@@ -8620,7 +8620,7 @@
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>0.211</v>
+        <v>0.217</v>
       </c>
       <c r="E2" s="5" t="inlineStr"/>
     </row>
@@ -8641,7 +8641,7 @@
         </is>
       </c>
       <c r="D3" s="5" t="n">
-        <v>0.039</v>
+        <v>0.04</v>
       </c>
       <c r="E3" s="5" t="inlineStr"/>
     </row>
@@ -8662,7 +8662,7 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>0.036</v>
+        <v>0.037</v>
       </c>
       <c r="E4" s="5" t="inlineStr"/>
     </row>
@@ -8683,7 +8683,7 @@
         </is>
       </c>
       <c r="D5" s="5" t="n">
-        <v>0.041</v>
+        <v>0.042</v>
       </c>
       <c r="E5" s="5" t="inlineStr"/>
     </row>
@@ -8704,7 +8704,7 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>0.04</v>
+        <v>0.035</v>
       </c>
       <c r="E6" s="5" t="inlineStr"/>
     </row>
@@ -8725,7 +8725,7 @@
         </is>
       </c>
       <c r="D7" s="5" t="n">
-        <v>0.04</v>
+        <v>0.037</v>
       </c>
       <c r="E7" s="5" t="inlineStr"/>
     </row>
@@ -8746,7 +8746,7 @@
         </is>
       </c>
       <c r="D8" s="5" t="n">
-        <v>0.06</v>
+        <v>0.058</v>
       </c>
       <c r="E8" s="5" t="inlineStr"/>
     </row>
@@ -8767,7 +8767,7 @@
         </is>
       </c>
       <c r="D9" s="5" t="n">
-        <v>0.055</v>
+        <v>0.047</v>
       </c>
       <c r="E9" s="5" t="inlineStr"/>
     </row>
@@ -8788,7 +8788,7 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>0.05</v>
+        <v>0.046</v>
       </c>
       <c r="E10" s="5" t="inlineStr"/>
     </row>
@@ -8809,7 +8809,7 @@
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>0.036</v>
+        <v>0.033</v>
       </c>
       <c r="E11" s="5" t="inlineStr"/>
     </row>
@@ -8830,7 +8830,7 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>0.036</v>
+        <v>0.035</v>
       </c>
       <c r="E12" s="5" t="inlineStr"/>
     </row>
@@ -8851,7 +8851,7 @@
         </is>
       </c>
       <c r="D13" s="5" t="n">
-        <v>0.057</v>
+        <v>0.058</v>
       </c>
       <c r="E13" s="5" t="inlineStr"/>
     </row>
@@ -8872,7 +8872,7 @@
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>0.067</v>
+        <v>0.065</v>
       </c>
       <c r="E14" s="5" t="inlineStr"/>
     </row>
@@ -8893,7 +8893,7 @@
         </is>
       </c>
       <c r="D15" s="5" t="n">
-        <v>0.034</v>
+        <v>0.038</v>
       </c>
       <c r="E15" s="5" t="inlineStr"/>
     </row>
@@ -8914,7 +8914,7 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>0.041</v>
+        <v>0.04</v>
       </c>
       <c r="E16" s="5" t="inlineStr"/>
     </row>
@@ -8935,7 +8935,7 @@
         </is>
       </c>
       <c r="D17" s="5" t="n">
-        <v>0.045</v>
+        <v>0.046</v>
       </c>
       <c r="E17" s="5" t="inlineStr"/>
     </row>
@@ -8956,7 +8956,7 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>0.036</v>
+        <v>0.037</v>
       </c>
       <c r="E18" s="5" t="inlineStr"/>
     </row>
@@ -8977,7 +8977,7 @@
         </is>
       </c>
       <c r="D19" s="5" t="n">
-        <v>0.033</v>
+        <v>0.035</v>
       </c>
       <c r="E19" s="5" t="inlineStr"/>
     </row>
@@ -8998,7 +8998,7 @@
         </is>
       </c>
       <c r="D20" s="5" t="n">
-        <v>0.033</v>
+        <v>0.032</v>
       </c>
       <c r="E20" s="5" t="inlineStr"/>
     </row>
@@ -9019,7 +9019,7 @@
         </is>
       </c>
       <c r="D21" s="5" t="n">
-        <v>0.038</v>
+        <v>0.029</v>
       </c>
       <c r="E21" s="5" t="inlineStr"/>
     </row>
@@ -9061,7 +9061,7 @@
         </is>
       </c>
       <c r="D23" s="5" t="n">
-        <v>0.03</v>
+        <v>0.028</v>
       </c>
       <c r="E23" s="5" t="inlineStr"/>
     </row>
@@ -9082,7 +9082,7 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>0.025</v>
+        <v>0.026</v>
       </c>
       <c r="E24" s="5" t="inlineStr"/>
     </row>
@@ -9103,7 +9103,7 @@
         </is>
       </c>
       <c r="D25" s="5" t="n">
-        <v>0.021</v>
+        <v>0.019</v>
       </c>
       <c r="E25" s="5" t="inlineStr"/>
     </row>
@@ -9124,7 +9124,7 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>0.03</v>
+        <v>0.029</v>
       </c>
       <c r="E26" s="5" t="inlineStr"/>
     </row>
@@ -9187,7 +9187,7 @@
         </is>
       </c>
       <c r="D29" s="5" t="n">
-        <v>0.037</v>
+        <v>0.035</v>
       </c>
       <c r="E29" s="5" t="inlineStr"/>
     </row>
@@ -9208,7 +9208,7 @@
         </is>
       </c>
       <c r="D30" s="5" t="n">
-        <v>0.019</v>
+        <v>0.016</v>
       </c>
       <c r="E30" s="5" t="inlineStr"/>
     </row>
@@ -9229,7 +9229,7 @@
         </is>
       </c>
       <c r="D31" s="5" t="n">
-        <v>0.02</v>
+        <v>0.026</v>
       </c>
       <c r="E31" s="5" t="inlineStr"/>
     </row>
@@ -9250,7 +9250,7 @@
         </is>
       </c>
       <c r="D32" s="5" t="n">
-        <v>0.025</v>
+        <v>0.026</v>
       </c>
       <c r="E32" s="5" t="inlineStr"/>
     </row>
@@ -9271,7 +9271,7 @@
         </is>
       </c>
       <c r="D33" s="5" t="n">
-        <v>0.017</v>
+        <v>0.018</v>
       </c>
       <c r="E33" s="5" t="inlineStr"/>
     </row>
@@ -9292,7 +9292,7 @@
         </is>
       </c>
       <c r="D34" s="5" t="n">
-        <v>0.025</v>
+        <v>0.021</v>
       </c>
       <c r="E34" s="5" t="inlineStr"/>
     </row>
@@ -9313,7 +9313,7 @@
         </is>
       </c>
       <c r="D35" s="5" t="n">
-        <v>0.023</v>
+        <v>0.022</v>
       </c>
       <c r="E35" s="5" t="inlineStr"/>
     </row>
@@ -9376,7 +9376,7 @@
         </is>
       </c>
       <c r="D38" s="5" t="n">
-        <v>0.022</v>
+        <v>0.021</v>
       </c>
       <c r="E38" s="5" t="inlineStr"/>
     </row>
@@ -9397,7 +9397,7 @@
         </is>
       </c>
       <c r="D39" s="5" t="n">
-        <v>0.016</v>
+        <v>0.019</v>
       </c>
       <c r="E39" s="5" t="inlineStr"/>
     </row>
@@ -9418,7 +9418,7 @@
         </is>
       </c>
       <c r="D40" s="5" t="n">
-        <v>0.125</v>
+        <v>0.131</v>
       </c>
       <c r="E40" s="5" t="inlineStr"/>
     </row>
@@ -9439,7 +9439,7 @@
         </is>
       </c>
       <c r="D41" s="5" t="n">
-        <v>0.023</v>
+        <v>0.022</v>
       </c>
       <c r="E41" s="5" t="inlineStr"/>
     </row>
@@ -9502,7 +9502,7 @@
         </is>
       </c>
       <c r="D44" s="5" t="n">
-        <v>0.104</v>
+        <v>0.047</v>
       </c>
       <c r="E44" s="5" t="inlineStr"/>
     </row>
@@ -9565,7 +9565,7 @@
         </is>
       </c>
       <c r="D47" s="5" t="n">
-        <v>0.021</v>
+        <v>0.02</v>
       </c>
       <c r="E47" s="5" t="inlineStr"/>
     </row>
@@ -9586,7 +9586,7 @@
         </is>
       </c>
       <c r="D48" s="5" t="n">
-        <v>0.019</v>
+        <v>0.017</v>
       </c>
       <c r="E48" s="5" t="inlineStr"/>
     </row>
@@ -9607,7 +9607,7 @@
         </is>
       </c>
       <c r="D49" s="5" t="n">
-        <v>0.019</v>
+        <v>0.017</v>
       </c>
       <c r="E49" s="5" t="inlineStr"/>
     </row>
@@ -9649,7 +9649,7 @@
         </is>
       </c>
       <c r="D51" s="5" t="n">
-        <v>0.019</v>
+        <v>0.02</v>
       </c>
       <c r="E51" s="5" t="inlineStr"/>
     </row>
@@ -9670,7 +9670,7 @@
         </is>
       </c>
       <c r="D52" s="5" t="n">
-        <v>0.019</v>
+        <v>0.024</v>
       </c>
       <c r="E52" s="5" t="inlineStr"/>
     </row>
@@ -9712,7 +9712,7 @@
         </is>
       </c>
       <c r="D54" s="5" t="n">
-        <v>0.02</v>
+        <v>0.019</v>
       </c>
       <c r="E54" s="5" t="inlineStr"/>
     </row>
@@ -9733,7 +9733,7 @@
         </is>
       </c>
       <c r="D55" s="5" t="n">
-        <v>0.019</v>
+        <v>0.021</v>
       </c>
       <c r="E55" s="5" t="inlineStr"/>
     </row>
@@ -9754,7 +9754,7 @@
         </is>
       </c>
       <c r="D56" s="5" t="n">
-        <v>0.022</v>
+        <v>0.017</v>
       </c>
       <c r="E56" s="5" t="inlineStr"/>
     </row>
@@ -9775,7 +9775,7 @@
         </is>
       </c>
       <c r="D57" s="5" t="n">
-        <v>0.017</v>
+        <v>0.018</v>
       </c>
       <c r="E57" s="5" t="inlineStr"/>
     </row>
@@ -9796,7 +9796,7 @@
         </is>
       </c>
       <c r="D58" s="5" t="n">
-        <v>0.02</v>
+        <v>0.019</v>
       </c>
       <c r="E58" s="5" t="inlineStr"/>
     </row>
@@ -9817,7 +9817,7 @@
         </is>
       </c>
       <c r="D59" s="5" t="n">
-        <v>0.018</v>
+        <v>0.02</v>
       </c>
       <c r="E59" s="5" t="inlineStr"/>
     </row>
@@ -9838,7 +9838,7 @@
         </is>
       </c>
       <c r="D60" s="5" t="n">
-        <v>0.017</v>
+        <v>0.018</v>
       </c>
       <c r="E60" s="5" t="inlineStr"/>
     </row>
@@ -9859,7 +9859,7 @@
         </is>
       </c>
       <c r="D61" s="5" t="n">
-        <v>0.018</v>
+        <v>0.017</v>
       </c>
       <c r="E61" s="5" t="inlineStr"/>
     </row>
@@ -9880,7 +9880,7 @@
         </is>
       </c>
       <c r="D62" s="5" t="n">
-        <v>0.016</v>
+        <v>0.017</v>
       </c>
       <c r="E62" s="5" t="inlineStr"/>
     </row>
@@ -9901,7 +9901,7 @@
         </is>
       </c>
       <c r="D63" s="5" t="n">
-        <v>0.017</v>
+        <v>0.018</v>
       </c>
       <c r="E63" s="5" t="inlineStr"/>
     </row>
@@ -9922,7 +9922,7 @@
         </is>
       </c>
       <c r="D64" s="5" t="n">
-        <v>0.016</v>
+        <v>0.017</v>
       </c>
       <c r="E64" s="5" t="inlineStr"/>
     </row>
@@ -9943,7 +9943,7 @@
         </is>
       </c>
       <c r="D65" s="5" t="n">
-        <v>0.018</v>
+        <v>0.022</v>
       </c>
       <c r="E65" s="5" t="inlineStr"/>
     </row>
@@ -9985,7 +9985,7 @@
         </is>
       </c>
       <c r="D67" s="5" t="n">
-        <v>0.016</v>
+        <v>0.018</v>
       </c>
       <c r="E67" s="5" t="inlineStr"/>
     </row>
@@ -10048,7 +10048,7 @@
         </is>
       </c>
       <c r="D70" s="5" t="n">
-        <v>0.019</v>
+        <v>0.02</v>
       </c>
       <c r="E70" s="5" t="inlineStr"/>
     </row>
@@ -10405,7 +10405,7 @@
         </is>
       </c>
       <c r="D87" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="E87" s="5" t="inlineStr"/>
     </row>
@@ -11014,7 +11014,7 @@
         </is>
       </c>
       <c r="D116" s="5" t="n">
-        <v>0.093</v>
+        <v>0.095</v>
       </c>
       <c r="E116" s="5" t="inlineStr"/>
     </row>
@@ -11035,7 +11035,7 @@
         </is>
       </c>
       <c r="D117" s="5" t="n">
-        <v>0.031</v>
+        <v>0.032</v>
       </c>
       <c r="E117" s="5" t="inlineStr"/>
     </row>
@@ -11077,7 +11077,7 @@
         </is>
       </c>
       <c r="D119" s="5" t="n">
-        <v>0.021</v>
+        <v>0.024</v>
       </c>
       <c r="E119" s="5" t="inlineStr"/>
     </row>
@@ -11119,7 +11119,7 @@
         </is>
       </c>
       <c r="D121" s="5" t="n">
-        <v>0.025</v>
+        <v>0.023</v>
       </c>
       <c r="E121" s="5" t="inlineStr"/>
     </row>
@@ -11140,7 +11140,7 @@
         </is>
       </c>
       <c r="D122" s="5" t="n">
-        <v>0.018</v>
+        <v>0.016</v>
       </c>
       <c r="E122" s="5" t="inlineStr"/>
     </row>
@@ -11182,7 +11182,7 @@
         </is>
       </c>
       <c r="D124" s="5" t="n">
-        <v>0.028</v>
+        <v>0.024</v>
       </c>
       <c r="E124" s="5" t="inlineStr"/>
     </row>
@@ -11266,7 +11266,7 @@
         </is>
       </c>
       <c r="D128" s="5" t="n">
-        <v>0.024</v>
+        <v>0.025</v>
       </c>
       <c r="E128" s="5" t="inlineStr"/>
     </row>
@@ -11287,7 +11287,7 @@
         </is>
       </c>
       <c r="D129" s="5" t="n">
-        <v>0.023</v>
+        <v>0.029</v>
       </c>
       <c r="E129" s="5" t="inlineStr"/>
     </row>
@@ -11392,7 +11392,7 @@
         </is>
       </c>
       <c r="D134" s="5" t="n">
-        <v>0.015</v>
+        <v>0.014</v>
       </c>
       <c r="E134" s="5" t="inlineStr"/>
     </row>
@@ -11434,7 +11434,7 @@
         </is>
       </c>
       <c r="D136" s="5" t="n">
-        <v>0.021</v>
+        <v>0.022</v>
       </c>
       <c r="E136" s="5" t="inlineStr"/>
     </row>
@@ -11455,7 +11455,7 @@
         </is>
       </c>
       <c r="D137" s="5" t="n">
-        <v>0.017</v>
+        <v>0.016</v>
       </c>
       <c r="E137" s="5" t="inlineStr"/>
     </row>
@@ -11476,7 +11476,7 @@
         </is>
       </c>
       <c r="D138" s="5" t="n">
-        <v>0.022</v>
+        <v>0.024</v>
       </c>
       <c r="E138" s="5" t="inlineStr"/>
     </row>
@@ -11497,7 +11497,7 @@
         </is>
       </c>
       <c r="D139" s="5" t="n">
-        <v>0.022</v>
+        <v>0.023</v>
       </c>
       <c r="E139" s="5" t="inlineStr"/>
     </row>
@@ -11938,7 +11938,7 @@
         </is>
       </c>
       <c r="D160" s="5" t="n">
-        <v>0.199</v>
+        <v>0.245</v>
       </c>
       <c r="E160" s="5" t="inlineStr"/>
     </row>
@@ -11959,7 +11959,7 @@
         </is>
       </c>
       <c r="D161" s="5" t="n">
-        <v>0.137</v>
+        <v>0.177</v>
       </c>
       <c r="E161" s="5" t="inlineStr"/>
     </row>
@@ -11980,7 +11980,7 @@
         </is>
       </c>
       <c r="D162" s="5" t="n">
-        <v>2.19</v>
+        <v>2.162</v>
       </c>
       <c r="E162" s="5" t="inlineStr"/>
     </row>
@@ -12001,7 +12001,7 @@
         </is>
       </c>
       <c r="D163" s="5" t="n">
-        <v>2.164</v>
+        <v>2.149</v>
       </c>
       <c r="E163" s="5" t="inlineStr"/>
     </row>
@@ -12022,7 +12022,7 @@
         </is>
       </c>
       <c r="D164" s="5" t="n">
-        <v>0.146</v>
+        <v>0.184</v>
       </c>
       <c r="E164" s="5" t="inlineStr"/>
     </row>
@@ -12043,7 +12043,7 @@
         </is>
       </c>
       <c r="D165" s="5" t="n">
-        <v>0.175</v>
+        <v>0.189</v>
       </c>
       <c r="E165" s="5" t="inlineStr"/>
     </row>
@@ -12064,7 +12064,7 @@
         </is>
       </c>
       <c r="D166" s="5" t="n">
-        <v>0.14</v>
+        <v>0.176</v>
       </c>
       <c r="E166" s="5" t="inlineStr"/>
     </row>
@@ -12127,7 +12127,7 @@
         </is>
       </c>
       <c r="D169" s="5" t="n">
-        <v>0.129</v>
+        <v>0.157</v>
       </c>
       <c r="E169" s="5" t="inlineStr"/>
     </row>
@@ -12148,7 +12148,7 @@
         </is>
       </c>
       <c r="D170" s="5" t="n">
-        <v>2.147</v>
+        <v>2.144</v>
       </c>
       <c r="E170" s="5" t="inlineStr"/>
     </row>
@@ -12190,7 +12190,7 @@
         </is>
       </c>
       <c r="D172" s="5" t="n">
-        <v>0.167</v>
+        <v>0.201</v>
       </c>
       <c r="E172" s="5" t="inlineStr"/>
     </row>
@@ -12211,7 +12211,7 @@
         </is>
       </c>
       <c r="D173" s="5" t="n">
-        <v>0.143</v>
+        <v>0.16</v>
       </c>
       <c r="E173" s="5" t="inlineStr"/>
     </row>
@@ -12232,7 +12232,7 @@
         </is>
       </c>
       <c r="D174" s="5" t="n">
-        <v>0.171</v>
+        <v>0.194</v>
       </c>
       <c r="E174" s="5" t="inlineStr"/>
     </row>
@@ -12253,7 +12253,7 @@
         </is>
       </c>
       <c r="D175" s="5" t="n">
-        <v>0.2</v>
+        <v>0.21</v>
       </c>
       <c r="E175" s="5" t="inlineStr"/>
     </row>
@@ -12295,7 +12295,7 @@
         </is>
       </c>
       <c r="D177" s="5" t="n">
-        <v>0.124</v>
+        <v>0.142</v>
       </c>
       <c r="E177" s="5" t="inlineStr"/>
     </row>
@@ -12316,7 +12316,7 @@
         </is>
       </c>
       <c r="D178" s="5" t="n">
-        <v>0.132</v>
+        <v>0.144</v>
       </c>
       <c r="E178" s="5" t="inlineStr"/>
     </row>
@@ -12337,7 +12337,7 @@
         </is>
       </c>
       <c r="D179" s="5" t="n">
-        <v>0.128</v>
+        <v>0.21</v>
       </c>
       <c r="E179" s="5" t="inlineStr"/>
     </row>
@@ -12379,7 +12379,7 @@
         </is>
       </c>
       <c r="D181" s="5" t="n">
-        <v>0.128</v>
+        <v>0.956</v>
       </c>
       <c r="E181" s="5" t="inlineStr"/>
     </row>
@@ -12400,7 +12400,7 @@
         </is>
       </c>
       <c r="D182" s="5" t="n">
-        <v>0.133</v>
+        <v>1.058</v>
       </c>
       <c r="E182" s="5" t="inlineStr"/>
     </row>
@@ -12421,7 +12421,7 @@
         </is>
       </c>
       <c r="D183" s="5" t="n">
-        <v>0.143</v>
+        <v>0.899</v>
       </c>
       <c r="E183" s="5" t="inlineStr"/>
     </row>
@@ -12442,7 +12442,7 @@
         </is>
       </c>
       <c r="D184" s="5" t="n">
-        <v>0.136</v>
+        <v>0.882</v>
       </c>
       <c r="E184" s="5" t="inlineStr"/>
     </row>
@@ -12463,7 +12463,7 @@
         </is>
       </c>
       <c r="D185" s="5" t="n">
-        <v>0.099</v>
+        <v>0.489</v>
       </c>
       <c r="E185" s="5" t="inlineStr"/>
     </row>
@@ -12484,7 +12484,7 @@
         </is>
       </c>
       <c r="D186" s="5" t="n">
-        <v>0.014</v>
+        <v>0.024</v>
       </c>
       <c r="E186" s="5" t="inlineStr"/>
     </row>
@@ -12505,7 +12505,7 @@
         </is>
       </c>
       <c r="D187" s="5" t="n">
-        <v>0.013</v>
+        <v>0.018</v>
       </c>
       <c r="E187" s="5" t="inlineStr"/>
     </row>
@@ -12526,7 +12526,7 @@
         </is>
       </c>
       <c r="D188" s="5" t="n">
-        <v>0.014</v>
+        <v>0.018</v>
       </c>
       <c r="E188" s="5" t="inlineStr"/>
     </row>
@@ -12547,7 +12547,7 @@
         </is>
       </c>
       <c r="D189" s="5" t="n">
-        <v>0.014</v>
+        <v>0.019</v>
       </c>
       <c r="E189" s="5" t="inlineStr"/>
     </row>
@@ -12589,7 +12589,7 @@
         </is>
       </c>
       <c r="D191" s="5" t="n">
-        <v>0.198</v>
+        <v>0.2</v>
       </c>
       <c r="E191" s="5" t="inlineStr"/>
     </row>
@@ -12610,7 +12610,7 @@
         </is>
       </c>
       <c r="D192" s="5" t="n">
-        <v>0.164</v>
+        <v>0.166</v>
       </c>
       <c r="E192" s="5" t="inlineStr"/>
     </row>
@@ -12631,7 +12631,7 @@
         </is>
       </c>
       <c r="D193" s="5" t="n">
-        <v>0.156</v>
+        <v>0.159</v>
       </c>
       <c r="E193" s="5" t="inlineStr"/>
     </row>
@@ -12652,7 +12652,7 @@
         </is>
       </c>
       <c r="D194" s="5" t="n">
-        <v>0.161</v>
+        <v>0.185</v>
       </c>
       <c r="E194" s="5" t="inlineStr"/>
     </row>
@@ -12736,7 +12736,7 @@
         </is>
       </c>
       <c r="D198" s="5" t="n">
-        <v>0.146</v>
+        <v>0.15</v>
       </c>
       <c r="E198" s="5" t="inlineStr"/>
     </row>
@@ -12820,7 +12820,7 @@
         </is>
       </c>
       <c r="D202" s="5" t="n">
-        <v>0.652</v>
+        <v>0.641</v>
       </c>
       <c r="E202" s="5" t="inlineStr"/>
     </row>
@@ -12841,7 +12841,7 @@
         </is>
       </c>
       <c r="D203" s="5" t="n">
-        <v>0.8070000000000001</v>
+        <v>0.715</v>
       </c>
       <c r="E203" s="5" t="inlineStr"/>
     </row>
@@ -12862,7 +12862,7 @@
         </is>
       </c>
       <c r="D204" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="E204" s="5" t="inlineStr"/>
     </row>
@@ -12883,7 +12883,7 @@
         </is>
       </c>
       <c r="D205" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="E205" s="5" t="inlineStr"/>
     </row>
@@ -12951,7 +12951,7 @@
         <v>800</v>
       </c>
       <c r="D2" s="5" t="n">
-        <v>591.49</v>
+        <v>582.62</v>
       </c>
       <c r="E2" s="5" t="inlineStr"/>
     </row>
@@ -12970,7 +12970,7 @@
         <v>10</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>139.82</v>
+        <v>149.52</v>
       </c>
       <c r="E3" s="5" t="inlineStr"/>
     </row>
@@ -13008,7 +13008,7 @@
         <v>724</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>6.19</v>
+        <v>6.1</v>
       </c>
       <c r="E5" s="5" t="inlineStr"/>
     </row>
@@ -13027,7 +13027,7 @@
         <v>7</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>140.93</v>
+        <v>149.73</v>
       </c>
       <c r="E6" s="5" t="inlineStr"/>
     </row>
@@ -13046,7 +13046,7 @@
         <v>7</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>594.09</v>
+        <v>579.75</v>
       </c>
       <c r="E7" s="5" t="inlineStr"/>
     </row>
@@ -13065,7 +13065,7 @@
         <v>368</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>84.70999999999999</v>
+        <v>82.86</v>
       </c>
       <c r="E8" s="5" t="inlineStr"/>
     </row>
@@ -13084,7 +13084,7 @@
         <v>36390</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>263.52</v>
+        <v>283.46</v>
       </c>
       <c r="E9" s="5" t="inlineStr"/>
     </row>
@@ -13103,7 +13103,7 @@
         <v>30</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>27.19</v>
+        <v>25.3</v>
       </c>
       <c r="E10" s="5" t="inlineStr"/>
     </row>
@@ -13122,7 +13122,7 @@
         <v>12401</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>108.79</v>
+        <v>106.56</v>
       </c>
       <c r="E11" s="5" t="inlineStr"/>
     </row>
@@ -13141,7 +13141,7 @@
         <v>12</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>4.3</v>
+        <v>4.56</v>
       </c>
       <c r="E12" s="5" t="inlineStr"/>
     </row>
@@ -13160,7 +13160,7 @@
         <v>800</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>133.97</v>
+        <v>132.13</v>
       </c>
       <c r="E13" s="5" t="inlineStr"/>
     </row>
@@ -13179,7 +13179,7 @@
         <v>136</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>228.01</v>
+        <v>231.69</v>
       </c>
       <c r="E14" s="5" t="inlineStr"/>
     </row>
@@ -13198,7 +13198,7 @@
         <v>800</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>225.81</v>
+        <v>226.82</v>
       </c>
       <c r="E15" s="5" t="inlineStr"/>
     </row>
@@ -13217,7 +13217,7 @@
         <v>2500</v>
       </c>
       <c r="D16" s="5" t="n">
-        <v>14.09</v>
+        <v>16.25</v>
       </c>
       <c r="E16" s="5" t="inlineStr"/>
     </row>
@@ -13236,7 +13236,7 @@
         <v>7</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>32.82</v>
+        <v>30.01</v>
       </c>
       <c r="E17" s="5" t="inlineStr"/>
     </row>
@@ -13255,7 +13255,7 @@
         <v>793</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>2.9</v>
+        <v>2.95</v>
       </c>
       <c r="E18" s="5" t="inlineStr"/>
     </row>
@@ -13274,7 +13274,7 @@
         <v>30</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>1.17</v>
+        <v>1.02</v>
       </c>
       <c r="E19" s="5" t="inlineStr"/>
     </row>
@@ -13293,7 +13293,7 @@
         <v>0</v>
       </c>
       <c r="D20" s="5" t="n">
-        <v>0.37</v>
+        <v>0.32</v>
       </c>
       <c r="E20" s="5" t="inlineStr"/>
     </row>
@@ -13312,7 +13312,7 @@
         <v>10</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>156</v>
+        <v>158.17</v>
       </c>
       <c r="E21" s="5" t="inlineStr"/>
     </row>
@@ -13331,7 +13331,7 @@
         <v>3082</v>
       </c>
       <c r="D22" s="5" t="n">
-        <v>55.05</v>
+        <v>53.81</v>
       </c>
       <c r="E22" s="5" t="inlineStr"/>
     </row>
@@ -13350,7 +13350,7 @@
         <v>6</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>5.31</v>
+        <v>6.04</v>
       </c>
       <c r="E23" s="5" t="inlineStr"/>
     </row>
@@ -13369,7 +13369,7 @@
         <v>368</v>
       </c>
       <c r="D24" s="5" t="n">
-        <v>82.14</v>
+        <v>86.69</v>
       </c>
       <c r="E24" s="5" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
fix(pages): add configure-pages step and base href for correct asset paths on /nova-payments-aml/
</commit_message>
<xml_diff>
--- a/08-qa-uat/matriz-ejecucion.xlsx
+++ b/08-qa-uat/matriz-ejecucion.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Casos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Matriz ejecucion" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cobertura" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Defectos" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Resultados pytest" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Controles SQL" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz ejecucion" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defectos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados pytest" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controles SQL" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Casos'!$A$1:$K$66</definedName>
@@ -567,7 +567,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29T02:16:36-03:00</t>
+          <t>2026-10-30T01:39:51-03:00</t>
         </is>
       </c>
     </row>
@@ -8620,7 +8620,7 @@
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>0.217</v>
+        <v>0.22</v>
       </c>
       <c r="E2" s="5" t="inlineStr"/>
     </row>
@@ -8641,7 +8641,7 @@
         </is>
       </c>
       <c r="D3" s="5" t="n">
-        <v>0.04</v>
+        <v>0.042</v>
       </c>
       <c r="E3" s="5" t="inlineStr"/>
     </row>
@@ -8704,7 +8704,7 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>0.035</v>
+        <v>0.04</v>
       </c>
       <c r="E6" s="5" t="inlineStr"/>
     </row>
@@ -8725,7 +8725,7 @@
         </is>
       </c>
       <c r="D7" s="5" t="n">
-        <v>0.037</v>
+        <v>0.045</v>
       </c>
       <c r="E7" s="5" t="inlineStr"/>
     </row>
@@ -8746,7 +8746,7 @@
         </is>
       </c>
       <c r="D8" s="5" t="n">
-        <v>0.058</v>
+        <v>0.061</v>
       </c>
       <c r="E8" s="5" t="inlineStr"/>
     </row>
@@ -8767,7 +8767,7 @@
         </is>
       </c>
       <c r="D9" s="5" t="n">
-        <v>0.047</v>
+        <v>0.049</v>
       </c>
       <c r="E9" s="5" t="inlineStr"/>
     </row>
@@ -8788,7 +8788,7 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>0.046</v>
+        <v>0.05</v>
       </c>
       <c r="E10" s="5" t="inlineStr"/>
     </row>
@@ -8809,7 +8809,7 @@
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>0.033</v>
+        <v>0.035</v>
       </c>
       <c r="E11" s="5" t="inlineStr"/>
     </row>
@@ -8851,7 +8851,7 @@
         </is>
       </c>
       <c r="D13" s="5" t="n">
-        <v>0.058</v>
+        <v>0.054</v>
       </c>
       <c r="E13" s="5" t="inlineStr"/>
     </row>
@@ -8872,7 +8872,7 @@
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>0.065</v>
+        <v>0.061</v>
       </c>
       <c r="E14" s="5" t="inlineStr"/>
     </row>
@@ -8893,7 +8893,7 @@
         </is>
       </c>
       <c r="D15" s="5" t="n">
-        <v>0.038</v>
+        <v>0.039</v>
       </c>
       <c r="E15" s="5" t="inlineStr"/>
     </row>
@@ -8914,7 +8914,7 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>0.04</v>
+        <v>0.041</v>
       </c>
       <c r="E16" s="5" t="inlineStr"/>
     </row>
@@ -8935,7 +8935,7 @@
         </is>
       </c>
       <c r="D17" s="5" t="n">
-        <v>0.046</v>
+        <v>0.044</v>
       </c>
       <c r="E17" s="5" t="inlineStr"/>
     </row>
@@ -8977,7 +8977,7 @@
         </is>
       </c>
       <c r="D19" s="5" t="n">
-        <v>0.035</v>
+        <v>0.036</v>
       </c>
       <c r="E19" s="5" t="inlineStr"/>
     </row>
@@ -8998,7 +8998,7 @@
         </is>
       </c>
       <c r="D20" s="5" t="n">
-        <v>0.032</v>
+        <v>0.041</v>
       </c>
       <c r="E20" s="5" t="inlineStr"/>
     </row>
@@ -9019,7 +9019,7 @@
         </is>
       </c>
       <c r="D21" s="5" t="n">
-        <v>0.029</v>
+        <v>0.045</v>
       </c>
       <c r="E21" s="5" t="inlineStr"/>
     </row>
@@ -9040,7 +9040,7 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>0.038</v>
+        <v>0.042</v>
       </c>
       <c r="E22" s="5" t="inlineStr"/>
     </row>
@@ -9061,7 +9061,7 @@
         </is>
       </c>
       <c r="D23" s="5" t="n">
-        <v>0.028</v>
+        <v>0.035</v>
       </c>
       <c r="E23" s="5" t="inlineStr"/>
     </row>
@@ -9082,7 +9082,7 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>0.026</v>
+        <v>0.028</v>
       </c>
       <c r="E24" s="5" t="inlineStr"/>
     </row>
@@ -9103,7 +9103,7 @@
         </is>
       </c>
       <c r="D25" s="5" t="n">
-        <v>0.019</v>
+        <v>0.018</v>
       </c>
       <c r="E25" s="5" t="inlineStr"/>
     </row>
@@ -9124,7 +9124,7 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>0.029</v>
+        <v>0.03</v>
       </c>
       <c r="E26" s="5" t="inlineStr"/>
     </row>
@@ -9187,7 +9187,7 @@
         </is>
       </c>
       <c r="D29" s="5" t="n">
-        <v>0.035</v>
+        <v>0.037</v>
       </c>
       <c r="E29" s="5" t="inlineStr"/>
     </row>
@@ -9229,7 +9229,7 @@
         </is>
       </c>
       <c r="D31" s="5" t="n">
-        <v>0.026</v>
+        <v>0.02</v>
       </c>
       <c r="E31" s="5" t="inlineStr"/>
     </row>
@@ -9271,7 +9271,7 @@
         </is>
       </c>
       <c r="D33" s="5" t="n">
-        <v>0.018</v>
+        <v>0.017</v>
       </c>
       <c r="E33" s="5" t="inlineStr"/>
     </row>
@@ -9313,7 +9313,7 @@
         </is>
       </c>
       <c r="D35" s="5" t="n">
-        <v>0.022</v>
+        <v>0.021</v>
       </c>
       <c r="E35" s="5" t="inlineStr"/>
     </row>
@@ -9355,7 +9355,7 @@
         </is>
       </c>
       <c r="D37" s="5" t="n">
-        <v>0.022</v>
+        <v>0.027</v>
       </c>
       <c r="E37" s="5" t="inlineStr"/>
     </row>
@@ -9376,7 +9376,7 @@
         </is>
       </c>
       <c r="D38" s="5" t="n">
-        <v>0.021</v>
+        <v>0.022</v>
       </c>
       <c r="E38" s="5" t="inlineStr"/>
     </row>
@@ -9397,7 +9397,7 @@
         </is>
       </c>
       <c r="D39" s="5" t="n">
-        <v>0.019</v>
+        <v>0.016</v>
       </c>
       <c r="E39" s="5" t="inlineStr"/>
     </row>
@@ -9418,7 +9418,7 @@
         </is>
       </c>
       <c r="D40" s="5" t="n">
-        <v>0.131</v>
+        <v>0.124</v>
       </c>
       <c r="E40" s="5" t="inlineStr"/>
     </row>
@@ -9460,7 +9460,7 @@
         </is>
       </c>
       <c r="D42" s="5" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
       <c r="E42" s="5" t="inlineStr"/>
     </row>
@@ -9502,7 +9502,7 @@
         </is>
       </c>
       <c r="D44" s="5" t="n">
-        <v>0.047</v>
+        <v>0.049</v>
       </c>
       <c r="E44" s="5" t="inlineStr"/>
     </row>
@@ -9586,7 +9586,7 @@
         </is>
       </c>
       <c r="D48" s="5" t="n">
-        <v>0.017</v>
+        <v>0.016</v>
       </c>
       <c r="E48" s="5" t="inlineStr"/>
     </row>
@@ -9628,7 +9628,7 @@
         </is>
       </c>
       <c r="D50" s="5" t="n">
-        <v>0.019</v>
+        <v>0.02</v>
       </c>
       <c r="E50" s="5" t="inlineStr"/>
     </row>
@@ -9649,7 +9649,7 @@
         </is>
       </c>
       <c r="D51" s="5" t="n">
-        <v>0.02</v>
+        <v>0.018</v>
       </c>
       <c r="E51" s="5" t="inlineStr"/>
     </row>
@@ -9670,7 +9670,7 @@
         </is>
       </c>
       <c r="D52" s="5" t="n">
-        <v>0.024</v>
+        <v>0.02</v>
       </c>
       <c r="E52" s="5" t="inlineStr"/>
     </row>
@@ -9691,7 +9691,7 @@
         </is>
       </c>
       <c r="D53" s="5" t="n">
-        <v>0.025</v>
+        <v>0.027</v>
       </c>
       <c r="E53" s="5" t="inlineStr"/>
     </row>
@@ -9712,7 +9712,7 @@
         </is>
       </c>
       <c r="D54" s="5" t="n">
-        <v>0.019</v>
+        <v>0.022</v>
       </c>
       <c r="E54" s="5" t="inlineStr"/>
     </row>
@@ -9733,7 +9733,7 @@
         </is>
       </c>
       <c r="D55" s="5" t="n">
-        <v>0.021</v>
+        <v>0.019</v>
       </c>
       <c r="E55" s="5" t="inlineStr"/>
     </row>
@@ -9754,7 +9754,7 @@
         </is>
       </c>
       <c r="D56" s="5" t="n">
-        <v>0.017</v>
+        <v>0.019</v>
       </c>
       <c r="E56" s="5" t="inlineStr"/>
     </row>
@@ -9775,7 +9775,7 @@
         </is>
       </c>
       <c r="D57" s="5" t="n">
-        <v>0.018</v>
+        <v>0.019</v>
       </c>
       <c r="E57" s="5" t="inlineStr"/>
     </row>
@@ -9796,7 +9796,7 @@
         </is>
       </c>
       <c r="D58" s="5" t="n">
-        <v>0.019</v>
+        <v>0.02</v>
       </c>
       <c r="E58" s="5" t="inlineStr"/>
     </row>
@@ -9838,7 +9838,7 @@
         </is>
       </c>
       <c r="D60" s="5" t="n">
-        <v>0.018</v>
+        <v>0.017</v>
       </c>
       <c r="E60" s="5" t="inlineStr"/>
     </row>
@@ -9859,7 +9859,7 @@
         </is>
       </c>
       <c r="D61" s="5" t="n">
-        <v>0.017</v>
+        <v>0.02</v>
       </c>
       <c r="E61" s="5" t="inlineStr"/>
     </row>
@@ -9880,7 +9880,7 @@
         </is>
       </c>
       <c r="D62" s="5" t="n">
-        <v>0.017</v>
+        <v>0.018</v>
       </c>
       <c r="E62" s="5" t="inlineStr"/>
     </row>
@@ -9901,7 +9901,7 @@
         </is>
       </c>
       <c r="D63" s="5" t="n">
-        <v>0.018</v>
+        <v>0.017</v>
       </c>
       <c r="E63" s="5" t="inlineStr"/>
     </row>
@@ -9922,7 +9922,7 @@
         </is>
       </c>
       <c r="D64" s="5" t="n">
-        <v>0.017</v>
+        <v>0.018</v>
       </c>
       <c r="E64" s="5" t="inlineStr"/>
     </row>
@@ -9943,7 +9943,7 @@
         </is>
       </c>
       <c r="D65" s="5" t="n">
-        <v>0.022</v>
+        <v>0.02</v>
       </c>
       <c r="E65" s="5" t="inlineStr"/>
     </row>
@@ -9964,7 +9964,7 @@
         </is>
       </c>
       <c r="D66" s="5" t="n">
-        <v>0.018</v>
+        <v>0.019</v>
       </c>
       <c r="E66" s="5" t="inlineStr"/>
     </row>
@@ -9985,7 +9985,7 @@
         </is>
       </c>
       <c r="D67" s="5" t="n">
-        <v>0.018</v>
+        <v>0.017</v>
       </c>
       <c r="E67" s="5" t="inlineStr"/>
     </row>
@@ -10006,7 +10006,7 @@
         </is>
       </c>
       <c r="D68" s="5" t="n">
-        <v>0.02</v>
+        <v>0.019</v>
       </c>
       <c r="E68" s="5" t="inlineStr"/>
     </row>
@@ -10027,7 +10027,7 @@
         </is>
       </c>
       <c r="D69" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="E69" s="5" t="inlineStr"/>
     </row>
@@ -10405,7 +10405,7 @@
         </is>
       </c>
       <c r="D87" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="E87" s="5" t="inlineStr"/>
     </row>
@@ -10426,7 +10426,7 @@
         </is>
       </c>
       <c r="D88" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E88" s="5" t="inlineStr"/>
     </row>
@@ -10447,7 +10447,7 @@
         </is>
       </c>
       <c r="D89" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E89" s="5" t="inlineStr"/>
     </row>
@@ -10468,7 +10468,7 @@
         </is>
       </c>
       <c r="D90" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E90" s="5" t="inlineStr"/>
     </row>
@@ -10489,7 +10489,7 @@
         </is>
       </c>
       <c r="D91" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E91" s="5" t="inlineStr"/>
     </row>
@@ -10531,7 +10531,7 @@
         </is>
       </c>
       <c r="D93" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E93" s="5" t="inlineStr"/>
     </row>
@@ -10552,7 +10552,7 @@
         </is>
       </c>
       <c r="D94" s="5" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
       <c r="E94" s="5" t="inlineStr"/>
     </row>
@@ -10573,7 +10573,7 @@
         </is>
       </c>
       <c r="D95" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E95" s="5" t="inlineStr"/>
     </row>
@@ -10762,7 +10762,7 @@
         </is>
       </c>
       <c r="D104" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E104" s="5" t="inlineStr"/>
     </row>
@@ -11014,7 +11014,7 @@
         </is>
       </c>
       <c r="D116" s="5" t="n">
-        <v>0.095</v>
+        <v>0.097</v>
       </c>
       <c r="E116" s="5" t="inlineStr"/>
     </row>
@@ -11035,7 +11035,7 @@
         </is>
       </c>
       <c r="D117" s="5" t="n">
-        <v>0.032</v>
+        <v>0.035</v>
       </c>
       <c r="E117" s="5" t="inlineStr"/>
     </row>
@@ -11056,7 +11056,7 @@
         </is>
       </c>
       <c r="D118" s="5" t="n">
-        <v>0.023</v>
+        <v>0.024</v>
       </c>
       <c r="E118" s="5" t="inlineStr"/>
     </row>
@@ -11077,7 +11077,7 @@
         </is>
       </c>
       <c r="D119" s="5" t="n">
-        <v>0.024</v>
+        <v>0.028</v>
       </c>
       <c r="E119" s="5" t="inlineStr"/>
     </row>
@@ -11140,7 +11140,7 @@
         </is>
       </c>
       <c r="D122" s="5" t="n">
-        <v>0.016</v>
+        <v>0.024</v>
       </c>
       <c r="E122" s="5" t="inlineStr"/>
     </row>
@@ -11161,7 +11161,7 @@
         </is>
       </c>
       <c r="D123" s="5" t="n">
-        <v>0.016</v>
+        <v>0.019</v>
       </c>
       <c r="E123" s="5" t="inlineStr"/>
     </row>
@@ -11182,7 +11182,7 @@
         </is>
       </c>
       <c r="D124" s="5" t="n">
-        <v>0.024</v>
+        <v>0.027</v>
       </c>
       <c r="E124" s="5" t="inlineStr"/>
     </row>
@@ -11245,7 +11245,7 @@
         </is>
       </c>
       <c r="D127" s="5" t="n">
-        <v>0.029</v>
+        <v>0.031</v>
       </c>
       <c r="E127" s="5" t="inlineStr"/>
     </row>
@@ -11266,7 +11266,7 @@
         </is>
       </c>
       <c r="D128" s="5" t="n">
-        <v>0.025</v>
+        <v>0.027</v>
       </c>
       <c r="E128" s="5" t="inlineStr"/>
     </row>
@@ -11287,7 +11287,7 @@
         </is>
       </c>
       <c r="D129" s="5" t="n">
-        <v>0.029</v>
+        <v>0.026</v>
       </c>
       <c r="E129" s="5" t="inlineStr"/>
     </row>
@@ -11308,7 +11308,7 @@
         </is>
       </c>
       <c r="D130" s="5" t="n">
-        <v>0.022</v>
+        <v>0.023</v>
       </c>
       <c r="E130" s="5" t="inlineStr"/>
     </row>
@@ -11329,7 +11329,7 @@
         </is>
       </c>
       <c r="D131" s="5" t="n">
-        <v>0.014</v>
+        <v>0.017</v>
       </c>
       <c r="E131" s="5" t="inlineStr"/>
     </row>
@@ -11350,7 +11350,7 @@
         </is>
       </c>
       <c r="D132" s="5" t="n">
-        <v>0.015</v>
+        <v>0.017</v>
       </c>
       <c r="E132" s="5" t="inlineStr"/>
     </row>
@@ -11371,7 +11371,7 @@
         </is>
       </c>
       <c r="D133" s="5" t="n">
-        <v>0.014</v>
+        <v>0.017</v>
       </c>
       <c r="E133" s="5" t="inlineStr"/>
     </row>
@@ -11392,7 +11392,7 @@
         </is>
       </c>
       <c r="D134" s="5" t="n">
-        <v>0.014</v>
+        <v>0.017</v>
       </c>
       <c r="E134" s="5" t="inlineStr"/>
     </row>
@@ -11413,7 +11413,7 @@
         </is>
       </c>
       <c r="D135" s="5" t="n">
-        <v>0.014</v>
+        <v>0.017</v>
       </c>
       <c r="E135" s="5" t="inlineStr"/>
     </row>
@@ -11434,7 +11434,7 @@
         </is>
       </c>
       <c r="D136" s="5" t="n">
-        <v>0.022</v>
+        <v>0.024</v>
       </c>
       <c r="E136" s="5" t="inlineStr"/>
     </row>
@@ -11455,7 +11455,7 @@
         </is>
       </c>
       <c r="D137" s="5" t="n">
-        <v>0.016</v>
+        <v>0.017</v>
       </c>
       <c r="E137" s="5" t="inlineStr"/>
     </row>
@@ -11476,7 +11476,7 @@
         </is>
       </c>
       <c r="D138" s="5" t="n">
-        <v>0.024</v>
+        <v>0.023</v>
       </c>
       <c r="E138" s="5" t="inlineStr"/>
     </row>
@@ -11938,7 +11938,7 @@
         </is>
       </c>
       <c r="D160" s="5" t="n">
-        <v>0.245</v>
+        <v>0.211</v>
       </c>
       <c r="E160" s="5" t="inlineStr"/>
     </row>
@@ -11959,7 +11959,7 @@
         </is>
       </c>
       <c r="D161" s="5" t="n">
-        <v>0.177</v>
+        <v>0.139</v>
       </c>
       <c r="E161" s="5" t="inlineStr"/>
     </row>
@@ -11980,7 +11980,7 @@
         </is>
       </c>
       <c r="D162" s="5" t="n">
-        <v>2.162</v>
+        <v>2.588</v>
       </c>
       <c r="E162" s="5" t="inlineStr"/>
     </row>
@@ -12001,7 +12001,7 @@
         </is>
       </c>
       <c r="D163" s="5" t="n">
-        <v>2.149</v>
+        <v>2.433</v>
       </c>
       <c r="E163" s="5" t="inlineStr"/>
     </row>
@@ -12022,7 +12022,7 @@
         </is>
       </c>
       <c r="D164" s="5" t="n">
-        <v>0.184</v>
+        <v>0.154</v>
       </c>
       <c r="E164" s="5" t="inlineStr"/>
     </row>
@@ -12043,7 +12043,7 @@
         </is>
       </c>
       <c r="D165" s="5" t="n">
-        <v>0.189</v>
+        <v>0.171</v>
       </c>
       <c r="E165" s="5" t="inlineStr"/>
     </row>
@@ -12064,7 +12064,7 @@
         </is>
       </c>
       <c r="D166" s="5" t="n">
-        <v>0.176</v>
+        <v>0.365</v>
       </c>
       <c r="E166" s="5" t="inlineStr"/>
     </row>
@@ -12127,7 +12127,7 @@
         </is>
       </c>
       <c r="D169" s="5" t="n">
-        <v>0.157</v>
+        <v>0.501</v>
       </c>
       <c r="E169" s="5" t="inlineStr"/>
     </row>
@@ -12148,7 +12148,7 @@
         </is>
       </c>
       <c r="D170" s="5" t="n">
-        <v>2.144</v>
+        <v>2.425</v>
       </c>
       <c r="E170" s="5" t="inlineStr"/>
     </row>
@@ -12190,7 +12190,7 @@
         </is>
       </c>
       <c r="D172" s="5" t="n">
-        <v>0.201</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="E172" s="5" t="inlineStr"/>
     </row>
@@ -12211,7 +12211,7 @@
         </is>
       </c>
       <c r="D173" s="5" t="n">
-        <v>0.16</v>
+        <v>0.39</v>
       </c>
       <c r="E173" s="5" t="inlineStr"/>
     </row>
@@ -12232,7 +12232,7 @@
         </is>
       </c>
       <c r="D174" s="5" t="n">
-        <v>0.194</v>
+        <v>0.175</v>
       </c>
       <c r="E174" s="5" t="inlineStr"/>
     </row>
@@ -12253,7 +12253,7 @@
         </is>
       </c>
       <c r="D175" s="5" t="n">
-        <v>0.21</v>
+        <v>0.193</v>
       </c>
       <c r="E175" s="5" t="inlineStr"/>
     </row>
@@ -12295,7 +12295,7 @@
         </is>
       </c>
       <c r="D177" s="5" t="n">
-        <v>0.142</v>
+        <v>0.133</v>
       </c>
       <c r="E177" s="5" t="inlineStr"/>
     </row>
@@ -12316,7 +12316,7 @@
         </is>
       </c>
       <c r="D178" s="5" t="n">
-        <v>0.144</v>
+        <v>0.122</v>
       </c>
       <c r="E178" s="5" t="inlineStr"/>
     </row>
@@ -12337,7 +12337,7 @@
         </is>
       </c>
       <c r="D179" s="5" t="n">
-        <v>0.21</v>
+        <v>0.126</v>
       </c>
       <c r="E179" s="5" t="inlineStr"/>
     </row>
@@ -12379,7 +12379,7 @@
         </is>
       </c>
       <c r="D181" s="5" t="n">
-        <v>0.956</v>
+        <v>0.127</v>
       </c>
       <c r="E181" s="5" t="inlineStr"/>
     </row>
@@ -12400,7 +12400,7 @@
         </is>
       </c>
       <c r="D182" s="5" t="n">
-        <v>1.058</v>
+        <v>0.132</v>
       </c>
       <c r="E182" s="5" t="inlineStr"/>
     </row>
@@ -12421,7 +12421,7 @@
         </is>
       </c>
       <c r="D183" s="5" t="n">
-        <v>0.899</v>
+        <v>0.145</v>
       </c>
       <c r="E183" s="5" t="inlineStr"/>
     </row>
@@ -12442,7 +12442,7 @@
         </is>
       </c>
       <c r="D184" s="5" t="n">
-        <v>0.882</v>
+        <v>0.13</v>
       </c>
       <c r="E184" s="5" t="inlineStr"/>
     </row>
@@ -12463,7 +12463,7 @@
         </is>
       </c>
       <c r="D185" s="5" t="n">
-        <v>0.489</v>
+        <v>0.112</v>
       </c>
       <c r="E185" s="5" t="inlineStr"/>
     </row>
@@ -12484,7 +12484,7 @@
         </is>
       </c>
       <c r="D186" s="5" t="n">
-        <v>0.024</v>
+        <v>0.014</v>
       </c>
       <c r="E186" s="5" t="inlineStr"/>
     </row>
@@ -12505,7 +12505,7 @@
         </is>
       </c>
       <c r="D187" s="5" t="n">
-        <v>0.018</v>
+        <v>0.014</v>
       </c>
       <c r="E187" s="5" t="inlineStr"/>
     </row>
@@ -12526,7 +12526,7 @@
         </is>
       </c>
       <c r="D188" s="5" t="n">
-        <v>0.018</v>
+        <v>0.014</v>
       </c>
       <c r="E188" s="5" t="inlineStr"/>
     </row>
@@ -12547,7 +12547,7 @@
         </is>
       </c>
       <c r="D189" s="5" t="n">
-        <v>0.019</v>
+        <v>0.016</v>
       </c>
       <c r="E189" s="5" t="inlineStr"/>
     </row>
@@ -12589,7 +12589,7 @@
         </is>
       </c>
       <c r="D191" s="5" t="n">
-        <v>0.2</v>
+        <v>0.231</v>
       </c>
       <c r="E191" s="5" t="inlineStr"/>
     </row>
@@ -12610,7 +12610,7 @@
         </is>
       </c>
       <c r="D192" s="5" t="n">
-        <v>0.166</v>
+        <v>0.177</v>
       </c>
       <c r="E192" s="5" t="inlineStr"/>
     </row>
@@ -12631,7 +12631,7 @@
         </is>
       </c>
       <c r="D193" s="5" t="n">
-        <v>0.159</v>
+        <v>0.17</v>
       </c>
       <c r="E193" s="5" t="inlineStr"/>
     </row>
@@ -12652,7 +12652,7 @@
         </is>
       </c>
       <c r="D194" s="5" t="n">
-        <v>0.185</v>
+        <v>0.172</v>
       </c>
       <c r="E194" s="5" t="inlineStr"/>
     </row>
@@ -12673,7 +12673,7 @@
         </is>
       </c>
       <c r="D195" s="5" t="n">
-        <v>0.004</v>
+        <v>0.007</v>
       </c>
       <c r="E195" s="5" t="inlineStr"/>
     </row>
@@ -12736,7 +12736,7 @@
         </is>
       </c>
       <c r="D198" s="5" t="n">
-        <v>0.15</v>
+        <v>0.176</v>
       </c>
       <c r="E198" s="5" t="inlineStr"/>
     </row>
@@ -12778,7 +12778,7 @@
         </is>
       </c>
       <c r="D200" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="E200" s="5" t="inlineStr"/>
     </row>
@@ -12820,7 +12820,7 @@
         </is>
       </c>
       <c r="D202" s="5" t="n">
-        <v>0.641</v>
+        <v>0.754</v>
       </c>
       <c r="E202" s="5" t="inlineStr"/>
     </row>
@@ -12841,7 +12841,7 @@
         </is>
       </c>
       <c r="D203" s="5" t="n">
-        <v>0.715</v>
+        <v>0.752</v>
       </c>
       <c r="E203" s="5" t="inlineStr"/>
     </row>
@@ -12883,7 +12883,7 @@
         </is>
       </c>
       <c r="D205" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E205" s="5" t="inlineStr"/>
     </row>
@@ -12951,7 +12951,7 @@
         <v>800</v>
       </c>
       <c r="D2" s="5" t="n">
-        <v>582.62</v>
+        <v>639.1</v>
       </c>
       <c r="E2" s="5" t="inlineStr"/>
     </row>
@@ -12970,7 +12970,7 @@
         <v>10</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>149.52</v>
+        <v>151.18</v>
       </c>
       <c r="E3" s="5" t="inlineStr"/>
     </row>
@@ -12989,7 +12989,7 @@
         <v>4</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>0.84</v>
+        <v>1.25</v>
       </c>
       <c r="E4" s="5" t="inlineStr"/>
     </row>
@@ -13008,7 +13008,7 @@
         <v>724</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>6.1</v>
+        <v>7.68</v>
       </c>
       <c r="E5" s="5" t="inlineStr"/>
     </row>
@@ -13027,7 +13027,7 @@
         <v>7</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>149.73</v>
+        <v>154.18</v>
       </c>
       <c r="E6" s="5" t="inlineStr"/>
     </row>
@@ -13043,10 +13043,10 @@
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>7</v>
+        <v>476</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>579.75</v>
+        <v>649.95</v>
       </c>
       <c r="E7" s="5" t="inlineStr"/>
     </row>
@@ -13062,10 +13062,10 @@
         </is>
       </c>
       <c r="C8" s="5" t="n">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>82.86</v>
+        <v>98.14</v>
       </c>
       <c r="E8" s="5" t="inlineStr"/>
     </row>
@@ -13081,10 +13081,10 @@
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>36390</v>
+        <v>36391</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>283.46</v>
+        <v>286.01</v>
       </c>
       <c r="E9" s="5" t="inlineStr"/>
     </row>
@@ -13103,7 +13103,7 @@
         <v>30</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>25.3</v>
+        <v>26.76</v>
       </c>
       <c r="E10" s="5" t="inlineStr"/>
     </row>
@@ -13119,10 +13119,10 @@
         </is>
       </c>
       <c r="C11" s="5" t="n">
-        <v>12401</v>
+        <v>12402</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>106.56</v>
+        <v>121.27</v>
       </c>
       <c r="E11" s="5" t="inlineStr"/>
     </row>
@@ -13141,7 +13141,7 @@
         <v>12</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>4.56</v>
+        <v>4.35</v>
       </c>
       <c r="E12" s="5" t="inlineStr"/>
     </row>
@@ -13160,7 +13160,7 @@
         <v>800</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>132.13</v>
+        <v>151.46</v>
       </c>
       <c r="E13" s="5" t="inlineStr"/>
     </row>
@@ -13179,7 +13179,7 @@
         <v>136</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>231.69</v>
+        <v>243.75</v>
       </c>
       <c r="E14" s="5" t="inlineStr"/>
     </row>
@@ -13198,7 +13198,7 @@
         <v>800</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>226.82</v>
+        <v>256.87</v>
       </c>
       <c r="E15" s="5" t="inlineStr"/>
     </row>
@@ -13217,7 +13217,7 @@
         <v>2500</v>
       </c>
       <c r="D16" s="5" t="n">
-        <v>16.25</v>
+        <v>16.61</v>
       </c>
       <c r="E16" s="5" t="inlineStr"/>
     </row>
@@ -13236,7 +13236,7 @@
         <v>7</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>30.01</v>
+        <v>31.91</v>
       </c>
       <c r="E17" s="5" t="inlineStr"/>
     </row>
@@ -13255,7 +13255,7 @@
         <v>793</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>2.95</v>
+        <v>4.3</v>
       </c>
       <c r="E18" s="5" t="inlineStr"/>
     </row>
@@ -13274,7 +13274,7 @@
         <v>30</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>1.02</v>
+        <v>1.19</v>
       </c>
       <c r="E19" s="5" t="inlineStr"/>
     </row>
@@ -13293,7 +13293,7 @@
         <v>0</v>
       </c>
       <c r="D20" s="5" t="n">
-        <v>0.32</v>
+        <v>0.51</v>
       </c>
       <c r="E20" s="5" t="inlineStr"/>
     </row>
@@ -13312,7 +13312,7 @@
         <v>10</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>158.17</v>
+        <v>171.35</v>
       </c>
       <c r="E21" s="5" t="inlineStr"/>
     </row>
@@ -13331,7 +13331,7 @@
         <v>3082</v>
       </c>
       <c r="D22" s="5" t="n">
-        <v>53.81</v>
+        <v>56.29</v>
       </c>
       <c r="E22" s="5" t="inlineStr"/>
     </row>
@@ -13350,7 +13350,7 @@
         <v>6</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>6.04</v>
+        <v>7.13</v>
       </c>
       <c r="E23" s="5" t="inlineStr"/>
     </row>
@@ -13366,10 +13366,10 @@
         </is>
       </c>
       <c r="C24" s="5" t="n">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="D24" s="5" t="n">
-        <v>86.69</v>
+        <v>94.42</v>
       </c>
       <c r="E24" s="5" t="inlineStr"/>
     </row>

</xml_diff>